<commit_message>
fix: 올리브영 chrome131->146 (Cloudflare 재차단) + 6/29 백필 + 6/30 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-06-29.xlsx
+++ b/data/daily/2026-06-29.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="올리브영" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -439,32 +428,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1093,32 +1082,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1430,6 +1419,360 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>상품명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[웰니스 루틴] 온리추얼 슬리밍컷 다이어트/리셋 브이라인/글로우업 콜라겐 7포(+1포)/14포 (8/14일분)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>온리추얼</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>11,900원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000236701&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CJ 한뿌리 흑삼지천보 진녹 30포 (1개월분) (온)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>한뿌리</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>250,000원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247763&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>피부/미용</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[10일콜라겐/모공,목주름/PDRN] 라이필 더마콜라겐 시그니처RN (10일분)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>라이필</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>15,840원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259411&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[6월 올영픽/골라담기] CJ웰케어 건강루틴 가격혁명 10종 택 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>씨제이웰케어</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5,900원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>프로뉴트리션</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>35,800원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000205496&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[포켓몬 에디션] 덴마크 유산균이야기 30캡슐 1+1 (+꼬부기 러기지택) (60일분)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>덴프스</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>30,400원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000206861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>피부/미용</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[6월 올영픽/윤광UP]온리추얼 글로우업 글루타치온 콜라겐 7포 (+1포 증정)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>온리추얼</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>15,900원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247570&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[6월 올영픽] 온리추얼 리셋 브이라인 7포 (+1포 증정) (8일분)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>온리추얼</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>14,900원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000249190&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[7월 올영픽] 오니스트 케라그로우 망고 14일 루틴 단품/기획(+2포)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>오니스트</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>28,900원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000241378&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[7월 올영픽] 식물성 멜라토닌 함유 멜라메이트 구미/로우슈가/버라이어티 구미 20/40/50구미</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>멜라메이트</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>13,000원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000223554&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1447,32 +1790,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1488,7 +1831,7 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>26.7</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
@@ -1510,7 +1853,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -1576,7 +1919,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -1620,7 +1963,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1639,10 +1982,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>23.3</v>
+        <v>22.5</v>
       </c>
       <c r="D9" t="n">
         <v>6</v>
@@ -1651,7 +1994,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1661,10 +2004,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -1673,7 +2016,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1683,10 +2026,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>6.7</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -1695,7 +2038,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1705,10 +2048,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>33.3</v>
+        <v>37.5</v>
       </c>
       <c r="D12" t="n">
         <v>3</v>
@@ -1717,7 +2060,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1727,7 +2070,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C13" t="n">
         <v>100</v>
@@ -1739,7 +2082,7 @@
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>